<commit_message>
feat: exclude representative names and titles from signature blocks in Web Preview and Excel Export
</commit_message>
<xml_diff>
--- a/source/TQC Database.xlsx
+++ b/source/TQC Database.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="86">
   <si>
     <t>key</t>
   </si>
@@ -91,57 +91,120 @@
     <t>id</t>
   </si>
   <si>
-    <t>mqfeu6zsb6mx8</t>
-  </si>
-  <si>
-    <t>Công ty Cổ phần Xây dựng Coteccons</t>
-  </si>
-  <si>
-    <t>Bolat Duisenov</t>
-  </si>
-  <si>
-    <t>Giám Đốc</t>
-  </si>
-  <si>
-    <t>Tòa nhà Coteccons, 236/6 Điện Biên Phủ, Phường 17, Quận Bình Thạnh, TP. Hồ Chí Minh</t>
-  </si>
-  <si>
-    <t>mqfev2ybjj16y</t>
-  </si>
-  <si>
-    <t>Công ty Cổ phần Tập đoàn Xây dựng Hòa Bình</t>
-  </si>
-  <si>
-    <t>Lê Viết Hải</t>
-  </si>
-  <si>
-    <t>Tòa nhà Pax Sky, 235 Võ Thị Sáu, Phường Võ Thị Sáu, Quận 3, TP. Hồ Chí Minh</t>
-  </si>
-  <si>
-    <t>mqff29wtf4nuj</t>
-  </si>
-  <si>
-    <t>Tổng Công ty Cổ phần Xuất nhập khẩu và Xây dựng Việt Nam (Vinaconex)</t>
-  </si>
-  <si>
-    <t>Nguyễn Xuân Đông</t>
-  </si>
-  <si>
-    <t>Tòa nhà Vinaconex, số 34 Láng Hạ, Phường Láng Hạ, Quận Đống Đa, Hà Nội</t>
-  </si>
-  <si>
-    <t>mqggiioyrhlbm</t>
+    <t>soHopDong</t>
+  </si>
+  <si>
+    <t>congTrinh</t>
+  </si>
+  <si>
+    <t>diaChiCongTrinh</t>
+  </si>
+  <si>
+    <t>soBBGT</t>
+  </si>
+  <si>
+    <t>soBBKL</t>
+  </si>
+  <si>
+    <t>hdNguyenTacSo</t>
+  </si>
+  <si>
+    <t>ngayKyHD</t>
+  </si>
+  <si>
+    <t>hoaDonSo</t>
+  </si>
+  <si>
+    <t>kyHieuHoaDon</t>
+  </si>
+  <si>
+    <t>ngayKyHoaDon</t>
+  </si>
+  <si>
+    <t>mqq9ye06bo3vt</t>
+  </si>
+  <si>
+    <t>Công ty TNHH Xây dựng Minh Phát</t>
+  </si>
+  <si>
+    <t>Nguyễn Văn Minh Phát</t>
+  </si>
+  <si>
+    <t>123 Lê Văn Lương, Q.7, TP.HCM</t>
+  </si>
+  <si>
+    <t>HĐ-001/2026</t>
+  </si>
+  <si>
+    <t>Nhà xưởng sản xuất Minh Phát</t>
+  </si>
+  <si>
+    <t>KCN Tân Đức, Long An</t>
+  </si>
+  <si>
+    <t>HĐNT-001/2026</t>
+  </si>
+  <si>
+    <t>AA/26E</t>
+  </si>
+  <si>
+    <t>mqq9zy0gc64qn</t>
+  </si>
+  <si>
+    <t>Công ty Cổ phần Đầu tư Xây dựng Hoàng Gia</t>
+  </si>
+  <si>
+    <t>Trần Quốc Hoàng</t>
+  </si>
+  <si>
+    <t>Tổng Giám đốc</t>
+  </si>
+  <si>
+    <t>45 Nguyễn Trãi, Q.1, TP.HCM</t>
+  </si>
+  <si>
+    <t>HĐ-002/2026</t>
+  </si>
+  <si>
+    <t>Chung cư Hoàng Gia Plaza</t>
+  </si>
+  <si>
+    <t>145 Nguyễn Văn Ngân, Thủ Đức, TP.HCM</t>
+  </si>
+  <si>
+    <t>HĐNT-002/2026</t>
+  </si>
+  <si>
+    <t>BB/26E</t>
+  </si>
+  <si>
+    <t>mqqacbxq5ttd2</t>
   </si>
   <si>
     <t>CÔNG TY CỔ PHẦN INDOCHINA BUILD VIỆT NAM</t>
   </si>
   <si>
-    <t>Nguyễn Thị Thùy Linh</t>
+    <t>Nguyễn Sỹ Dũng</t>
+  </si>
+  <si>
+    <t>Chỉ Huy Trưởng</t>
   </si>
   <si>
     <t>Ô CN6 - KCN Nguyên Khê - Xã Phúc Thịnh  – TP. Hà Nội</t>
   </si>
   <si>
+    <t>Khu liên hợp xử lý chất thải rắn Khánh Sơn</t>
+  </si>
+  <si>
+    <t>Đường Hoàng Văn Thái, Phường Hoà Khánh, Thành phố Đà Nẵng</t>
+  </si>
+  <si>
+    <t>584/2025/HĐNT/ICB- TQC</t>
+  </si>
+  <si>
+    <t>HĐ123</t>
+  </si>
+  <si>
     <t>ten</t>
   </si>
   <si>
@@ -172,12 +235,15 @@
     <t>mqg3thca79za0</t>
   </si>
   <si>
+    <t>Đá 5x5</t>
+  </si>
+  <si>
+    <t>mqg3u1bkhtmpc</t>
+  </si>
+  <si>
     <t>Đá 1x2</t>
   </si>
   <si>
-    <t>mqg3u1bkhtmpc</t>
-  </si>
-  <si>
     <t>ngay</t>
   </si>
   <si>
@@ -199,49 +265,19 @@
     <t>ghiChu</t>
   </si>
   <si>
-    <t>mqfflv63cozop</t>
-  </si>
-  <si>
-    <t>92B-123456</t>
-  </si>
-  <si>
-    <t>mqffrislo4br0</t>
-  </si>
-  <si>
-    <t>mqffvaeuo5hve</t>
-  </si>
-  <si>
-    <t>92H-02587</t>
-  </si>
-  <si>
-    <t>mqg0le7yihk9r</t>
-  </si>
-  <si>
-    <t>92H-202020</t>
-  </si>
-  <si>
-    <t>mqg1winylwvu8</t>
-  </si>
-  <si>
-    <t>TEST</t>
-  </si>
-  <si>
-    <t>mqg4gql4se1ui</t>
-  </si>
-  <si>
-    <t>mqgab49geslz4</t>
-  </si>
-  <si>
-    <t>92H-1111</t>
-  </si>
-  <si>
-    <t>mqgabkmffmc89</t>
-  </si>
-  <si>
-    <t>92H-3333</t>
-  </si>
-  <si>
-    <t>mqgacw0op4gft</t>
+    <t>mqqa3hzq4n0hn</t>
+  </si>
+  <si>
+    <t>mqqa3ua5gyo4w</t>
+  </si>
+  <si>
+    <t>92C-22169</t>
+  </si>
+  <si>
+    <t>mqqa43je7vgii</t>
+  </si>
+  <si>
+    <t>43H-06831</t>
   </si>
 </sst>
 </file>
@@ -300,10 +336,10 @@
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="11" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
@@ -684,85 +720,164 @@
       <c r="F1" s="1" t="s">
         <v>10</v>
       </c>
+      <c r="G1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>32</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>23</v>
+        <v>33</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>24</v>
+        <v>34</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>26</v>
+        <v>7</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>27</v>
+        <v>36</v>
       </c>
       <c r="F2" s="2">
-        <v>3.03443233E8</v>
+        <v>3.14567891E8</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="M2" s="3">
+        <v>46162.0</v>
+      </c>
+      <c r="N2" s="2">
+        <v>123.0</v>
+      </c>
+      <c r="O2" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="P2" s="3">
+        <v>46162.0</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>28</v>
+        <v>42</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>29</v>
+        <v>43</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>30</v>
+        <v>44</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>26</v>
+        <v>45</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>31</v>
+        <v>46</v>
       </c>
       <c r="F3" s="2">
-        <v>3.02158498E8</v>
+        <v>3.19876543E8</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="L3" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="M3" s="3">
+        <v>46168.0</v>
+      </c>
+      <c r="N3" s="2">
+        <v>456.0</v>
+      </c>
+      <c r="O3" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="P3" s="3">
+        <v>46168.0</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>32</v>
+        <v>52</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>33</v>
+        <v>53</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>34</v>
+        <v>54</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>26</v>
+        <v>55</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>35</v>
+        <v>56</v>
       </c>
       <c r="F4" s="2">
-        <v>1.00105616E8</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="F5" s="2">
         <v>1.04835204E8</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="L4" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="M4" s="3">
+        <v>45910.0</v>
+      </c>
+      <c r="N4" s="2">
+        <v>123456.0</v>
+      </c>
+      <c r="O4" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="P4" s="3">
+        <v>46196.0</v>
       </c>
     </row>
   </sheetData>
@@ -785,83 +900,83 @@
         <v>22</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>40</v>
+        <v>61</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>41</v>
+        <v>62</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>42</v>
+        <v>63</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>43</v>
+        <v>64</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>44</v>
+        <v>65</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>45</v>
+        <v>66</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="D2" s="3">
+        <v>67</v>
+      </c>
+      <c r="D2" s="4">
         <v>355000.0</v>
       </c>
-      <c r="E2" s="3">
+      <c r="E2" s="4">
         <v>115000.0</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>47</v>
+        <v>68</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>48</v>
+        <v>69</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="D3" s="3">
+        <v>67</v>
+      </c>
+      <c r="D3" s="4">
         <v>220000.0</v>
       </c>
-      <c r="E3" s="3">
+      <c r="E3" s="4">
         <v>100000.0</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>49</v>
+        <v>70</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>50</v>
+        <v>71</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="D4" s="3">
+        <v>67</v>
+      </c>
+      <c r="D4" s="4">
         <v>200000.0</v>
       </c>
-      <c r="E4" s="3">
+      <c r="E4" s="4">
         <v>110000.0</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>51</v>
+        <v>72</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>50</v>
+        <v>73</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="D5" s="3">
+        <v>67</v>
+      </c>
+      <c r="D5" s="4">
         <v>250000.0</v>
       </c>
-      <c r="E5" s="3">
+      <c r="E5" s="4">
         <v>125000.0</v>
       </c>
     </row>
@@ -885,235 +1000,94 @@
         <v>22</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>52</v>
+        <v>74</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>53</v>
+        <v>75</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>55</v>
+        <v>77</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>56</v>
+        <v>78</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>57</v>
+        <v>79</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>58</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="B2" s="4">
-        <v>46174.0</v>
-      </c>
-      <c r="C2" s="5" t="s">
-        <v>60</v>
-      </c>
-      <c r="D2" s="3">
+        <v>81</v>
+      </c>
+      <c r="B2" s="3">
+        <v>46196.0</v>
+      </c>
+      <c r="C2" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="D2" s="4">
         <v>1.0</v>
       </c>
-      <c r="E2" s="3">
+      <c r="E2" s="4">
         <v>20.0</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>23</v>
+        <v>52</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>44</v>
+        <v>70</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="B3" s="4">
-        <v>46174.0</v>
-      </c>
-      <c r="C3" s="5" t="s">
-        <v>60</v>
-      </c>
-      <c r="D3" s="3">
-        <v>3.0</v>
-      </c>
-      <c r="E3" s="3">
-        <v>23.0</v>
+        <v>82</v>
+      </c>
+      <c r="B3" s="3">
+        <v>46195.0</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="D3" s="4">
+        <v>1.0</v>
+      </c>
+      <c r="E3" s="4">
+        <v>33.0</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>23</v>
+        <v>52</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>44</v>
+        <v>70</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="B4" s="4">
-        <v>46174.0</v>
+        <v>84</v>
+      </c>
+      <c r="B4" s="3">
+        <v>46196.0</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="D4" s="3">
+        <v>85</v>
+      </c>
+      <c r="D4" s="4">
         <v>1.0</v>
       </c>
-      <c r="E4" s="3">
-        <v>16.0</v>
+      <c r="E4" s="4">
+        <v>44.0</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>23</v>
+        <v>52</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="B5" s="4">
-        <v>46179.0</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="D5" s="3">
-        <v>5.0</v>
-      </c>
-      <c r="E5" s="3">
-        <v>100.0</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="G5" s="2" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="B6" s="4">
-        <v>46190.0</v>
-      </c>
-      <c r="C6" s="5">
-        <v>0.0</v>
-      </c>
-      <c r="D6" s="3">
-        <v>1.0</v>
-      </c>
-      <c r="E6" s="3">
-        <v>55.0</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="G6" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="H6" s="2" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="s">
         <v>68</v>
-      </c>
-      <c r="B7" s="4">
-        <v>46189.0</v>
-      </c>
-      <c r="C7" s="5">
-        <v>0.0</v>
-      </c>
-      <c r="D7" s="3">
-        <v>1.0</v>
-      </c>
-      <c r="E7" s="3">
-        <v>66.0</v>
-      </c>
-      <c r="F7" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="G7" s="2" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="B8" s="4">
-        <v>46189.0</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="D8" s="3">
-        <v>1.0</v>
-      </c>
-      <c r="E8" s="3">
-        <v>44.0</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="G8" s="2" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="B9" s="4">
-        <v>46189.0</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="D9" s="3">
-        <v>1.0</v>
-      </c>
-      <c r="E9" s="3">
-        <v>88.7</v>
-      </c>
-      <c r="F9" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="G9" s="2" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="B10" s="4">
-        <v>46189.0</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="D10" s="3">
-        <v>3.0</v>
-      </c>
-      <c r="E10" s="3">
-        <v>50.5</v>
-      </c>
-      <c r="F10" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="G10" s="2" t="s">
-        <v>47</v>
       </c>
     </row>
   </sheetData>

</xml_diff>